<commit_message>
Fix: 支持设置 sheet tab color
</commit_message>
<xml_diff>
--- a/src/test/resources/test.xlsx
+++ b/src/test/resources/test.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="7270" activeTab="2"/>
+    <workbookView windowWidth="20752" windowHeight="9105"/>
   </bookViews>
   <sheets>
     <sheet name="bak" sheetId="5" r:id="rId1"/>
@@ -20,7 +20,20 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sheet1!$A$1:$G$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Sheet1 (2)'!$A$1:$H$35</definedName>
   </definedNames>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -218,7 +231,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
@@ -242,34 +255,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
@@ -283,14 +268,6 @@
       <color rgb="FF800080"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -330,6 +307,21 @@
       <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="宋体"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -380,7 +372,28 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FF9C6500"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -431,7 +444,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
+        <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -443,7 +456,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -455,13 +480,43 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
+        <fgColor rgb="FFFFEB9C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -473,7 +528,43 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -485,37 +576,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -527,60 +588,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -594,6 +601,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -640,21 +653,6 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
         <color rgb="FFB2B2B2"/>
       </left>
       <right style="thin">
@@ -683,6 +681,21 @@
       <top/>
       <bottom style="medium">
         <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -741,148 +754,148 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="17" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="17" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="18" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1043,52 +1056,52 @@
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="货币[0]" xfId="1" builtinId="7"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="2" builtinId="38"/>
-    <cellStyle name="输入" xfId="3" builtinId="20"/>
-    <cellStyle name="货币" xfId="4" builtinId="4"/>
-    <cellStyle name="千位分隔[0]" xfId="5" builtinId="6"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="6" builtinId="39"/>
-    <cellStyle name="差" xfId="7" builtinId="27"/>
-    <cellStyle name="千位分隔" xfId="8" builtinId="3"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="9" builtinId="40"/>
-    <cellStyle name="超链接" xfId="10" builtinId="8"/>
-    <cellStyle name="百分比" xfId="11" builtinId="5"/>
-    <cellStyle name="已访问的超链接" xfId="12" builtinId="9"/>
-    <cellStyle name="注释" xfId="13" builtinId="10"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="14" builtinId="36"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
     <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="警告文本" xfId="16" builtinId="11"/>
-    <cellStyle name="标题" xfId="17" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="18" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="19" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="20" builtinId="17"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="21" builtinId="32"/>
-    <cellStyle name="标题 3" xfId="22" builtinId="18"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="23" builtinId="44"/>
-    <cellStyle name="输出" xfId="24" builtinId="21"/>
-    <cellStyle name="计算" xfId="25" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="26" builtinId="23"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="27" builtinId="50"/>
-    <cellStyle name="强调文字颜色 2" xfId="28" builtinId="33"/>
-    <cellStyle name="链接单元格" xfId="29" builtinId="24"/>
-    <cellStyle name="汇总" xfId="30" builtinId="25"/>
-    <cellStyle name="好" xfId="31" builtinId="26"/>
-    <cellStyle name="适中" xfId="32" builtinId="28"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="33" builtinId="46"/>
-    <cellStyle name="强调文字颜色 1" xfId="34" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="35" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="36" builtinId="31"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="37" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="38" builtinId="35"/>
-    <cellStyle name="强调文字颜色 3" xfId="39" builtinId="37"/>
-    <cellStyle name="强调文字颜色 4" xfId="40" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="41" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="42" builtinId="43"/>
-    <cellStyle name="强调文字颜色 5" xfId="43" builtinId="45"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="44" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="45" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="46" builtinId="49"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
     <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
@@ -1387,27 +1400,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+  <sheetPr>
+    <tabColor rgb="FFFF0000"/>
+  </sheetPr>
   <dimension ref="A1:J64"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="31.4454545454545" customWidth="1"/>
+    <col min="1" max="1" width="31.4424778761062" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="4" width="27.1090909090909" customWidth="1"/>
-    <col min="5" max="5" width="18.3363636363636" customWidth="1"/>
-    <col min="6" max="6" width="18.6636363636364" customWidth="1"/>
-    <col min="7" max="7" width="17.5545454545455" customWidth="1"/>
-    <col min="8" max="8" width="9.66363636363636" customWidth="1"/>
-    <col min="9" max="9" width="64.5545454545454" customWidth="1"/>
-    <col min="10" max="10" width="39.6636363636364" customWidth="1"/>
+    <col min="3" max="4" width="27.1061946902655" customWidth="1"/>
+    <col min="5" max="5" width="18.3362831858407" customWidth="1"/>
+    <col min="6" max="6" width="18.6637168141593" customWidth="1"/>
+    <col min="7" max="7" width="17.5575221238938" customWidth="1"/>
+    <col min="8" max="8" width="9.66371681415929" customWidth="1"/>
+    <col min="9" max="9" width="64.5575221238938" customWidth="1"/>
+    <col min="10" max="10" width="39.6637168141593" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:9">
       <c r="A1" s="16">
         <v>34543</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:9">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -1433,7 +1448,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:9">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -1452,7 +1467,7 @@
       </c>
       <c r="G3" s="9"/>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:9">
       <c r="A4" s="11">
         <v>0</v>
       </c>
@@ -1471,7 +1486,7 @@
       </c>
       <c r="G4" s="9"/>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:9">
       <c r="A5" s="5"/>
       <c r="B5" s="6">
         <v>45007</v>
@@ -1488,7 +1503,7 @@
       </c>
       <c r="G5" s="9"/>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:9">
       <c r="A6" s="15"/>
       <c r="B6" s="42">
         <v>45007</v>
@@ -1505,7 +1520,7 @@
       </c>
       <c r="G6" s="9"/>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:9">
       <c r="A7" s="16"/>
       <c r="B7" s="16" t="s">
         <v>10</v>
@@ -1518,7 +1533,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:9">
       <c r="A8" s="43"/>
       <c r="B8" s="42">
         <v>45007</v>
@@ -1535,7 +1550,7 @@
       </c>
       <c r="G8" s="9"/>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:9">
       <c r="A9" s="11"/>
       <c r="B9" s="14">
         <v>45030</v>
@@ -1552,7 +1567,7 @@
       </c>
       <c r="G9" s="13"/>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:9">
       <c r="A10" s="11"/>
       <c r="B10" s="14"/>
       <c r="C10" s="13" t="s">
@@ -1563,7 +1578,7 @@
       <c r="F10" s="50"/>
       <c r="G10" s="13"/>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:9">
       <c r="A11" s="11"/>
       <c r="B11" s="14"/>
       <c r="C11" s="13" t="s">
@@ -1574,7 +1589,7 @@
       <c r="F11" s="50"/>
       <c r="G11" s="13"/>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:9">
       <c r="A12" s="11"/>
       <c r="B12" s="14"/>
       <c r="C12" s="13" t="s">
@@ -1595,7 +1610,7 @@
       <c r="G13" s="13"/>
       <c r="I13" s="9"/>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:9">
       <c r="A14" s="11"/>
       <c r="B14" s="14"/>
       <c r="C14" s="13"/>
@@ -1604,7 +1619,7 @@
       <c r="F14" s="50"/>
       <c r="G14" s="13"/>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:9">
       <c r="A15" s="11"/>
       <c r="B15" s="14"/>
       <c r="C15" s="13"/>
@@ -1613,7 +1628,7 @@
       <c r="F15" s="50"/>
       <c r="G15" s="13"/>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:9">
       <c r="A16" s="11"/>
       <c r="B16" s="14">
         <v>45016</v>
@@ -1630,7 +1645,7 @@
       </c>
       <c r="G16" s="9"/>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:10">
       <c r="A17" s="11"/>
       <c r="B17" s="14">
         <v>45027</v>
@@ -1647,7 +1662,7 @@
       </c>
       <c r="G17" s="9"/>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:10">
       <c r="A18" s="11"/>
       <c r="B18" s="14">
         <v>45020</v>
@@ -1664,7 +1679,7 @@
       </c>
       <c r="G18" s="9"/>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:10">
       <c r="A19" s="16"/>
       <c r="B19" s="16" t="s">
         <v>10</v>
@@ -1677,7 +1692,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:10">
       <c r="A20" s="44"/>
       <c r="B20" s="14">
         <v>45007</v>
@@ -1695,7 +1710,7 @@
       <c r="G20" s="26"/>
       <c r="I20" s="45"/>
     </row>
-    <row r="21" spans="1:9">
+    <row r="21" spans="1:10">
       <c r="A21" s="11"/>
       <c r="B21" s="14"/>
       <c r="C21" s="13" t="s">
@@ -1709,7 +1724,7 @@
       <c r="G21" s="26"/>
       <c r="I21" s="45"/>
     </row>
-    <row r="22" spans="1:9">
+    <row r="22" spans="1:10">
       <c r="A22" s="11"/>
       <c r="B22" s="14"/>
       <c r="C22" s="13" t="s">
@@ -1723,7 +1738,7 @@
       <c r="G22" s="26"/>
       <c r="I22" s="45"/>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:10">
       <c r="A23" s="11"/>
       <c r="B23" s="14"/>
       <c r="C23" s="13" t="s">
@@ -1737,7 +1752,7 @@
       <c r="G23" s="26"/>
       <c r="I23" s="45"/>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:10">
       <c r="A24" s="11"/>
       <c r="B24" s="14"/>
       <c r="C24" s="13" t="s">
@@ -1751,7 +1766,7 @@
       <c r="G24" s="26"/>
       <c r="I24" s="45"/>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:10">
       <c r="A25" s="11"/>
       <c r="B25" s="14"/>
       <c r="C25" s="13" t="s">
@@ -1765,7 +1780,7 @@
       <c r="G25" s="26"/>
       <c r="I25" s="45"/>
     </row>
-    <row r="26" spans="1:9">
+    <row r="26" spans="1:10">
       <c r="A26" s="11"/>
       <c r="B26" s="14"/>
       <c r="C26" s="13"/>
@@ -2092,7 +2107,7 @@
       <c r="I47" s="45"/>
       <c r="J47" s="47"/>
     </row>
-    <row r="48" spans="1:7">
+    <row r="48" spans="1:10">
       <c r="A48" s="5"/>
       <c r="B48" s="6">
         <v>45007</v>
@@ -2322,7 +2337,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:G64">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A2:G64" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2335,20 +2350,20 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:J30"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="31.4454545454545" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="31.4424778761062" hidden="1" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="4" width="27.1090909090909" customWidth="1"/>
-    <col min="5" max="5" width="18.3363636363636" customWidth="1"/>
-    <col min="6" max="6" width="18.6636363636364" customWidth="1"/>
-    <col min="7" max="7" width="17.5545454545455" customWidth="1"/>
-    <col min="8" max="8" width="9.66363636363636" customWidth="1"/>
-    <col min="9" max="9" width="64.5545454545454" customWidth="1"/>
-    <col min="10" max="10" width="39.6636363636364" customWidth="1"/>
+    <col min="3" max="4" width="27.1061946902655" customWidth="1"/>
+    <col min="5" max="5" width="18.3362831858407" customWidth="1"/>
+    <col min="6" max="6" width="18.6637168141593" customWidth="1"/>
+    <col min="7" max="7" width="17.5575221238938" customWidth="1"/>
+    <col min="8" max="8" width="9.66371681415929" customWidth="1"/>
+    <col min="9" max="9" width="64.5575221238938" customWidth="1"/>
+    <col min="10" max="10" width="39.6637168141593" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:10">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2374,7 +2389,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:10">
       <c r="A2" s="5"/>
       <c r="B2" s="6">
         <v>44988</v>
@@ -2389,7 +2404,7 @@
       <c r="F2" s="7"/>
       <c r="G2" s="9"/>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:10">
       <c r="A3" s="11"/>
       <c r="B3" s="6">
         <v>45016</v>
@@ -2404,7 +2419,7 @@
       <c r="F3" s="7"/>
       <c r="G3" s="9"/>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:10">
       <c r="A4" s="5"/>
       <c r="B4" s="6">
         <v>45007</v>
@@ -2419,7 +2434,7 @@
       <c r="F4" s="7"/>
       <c r="G4" s="9"/>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:10">
       <c r="A5" s="15"/>
       <c r="B5" s="42">
         <v>45007</v>
@@ -2434,7 +2449,7 @@
       <c r="F5" s="15"/>
       <c r="G5" s="9"/>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:10">
       <c r="A6" s="16"/>
       <c r="B6" s="16" t="s">
         <v>10</v>
@@ -2447,7 +2462,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:10">
       <c r="A7" s="43"/>
       <c r="B7" s="42">
         <v>45007</v>
@@ -2462,7 +2477,7 @@
       <c r="F7" s="15"/>
       <c r="G7" s="9"/>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:10">
       <c r="A8" s="11"/>
       <c r="B8" s="14">
         <v>45030</v>
@@ -2477,7 +2492,7 @@
       <c r="F8" s="13"/>
       <c r="G8" s="13"/>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:10">
       <c r="A9" s="11"/>
       <c r="B9" s="14">
         <v>45016</v>
@@ -2492,7 +2507,7 @@
       <c r="F9" s="13"/>
       <c r="G9" s="9"/>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:10">
       <c r="A10" s="11"/>
       <c r="B10" s="14">
         <v>45027</v>
@@ -2507,7 +2522,7 @@
       <c r="F10" s="13"/>
       <c r="G10" s="9"/>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:10">
       <c r="A11" s="11"/>
       <c r="B11" s="14">
         <v>45020</v>
@@ -2522,7 +2537,7 @@
       <c r="F11" s="13"/>
       <c r="G11" s="9"/>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:10">
       <c r="A12" s="16"/>
       <c r="B12" s="16" t="s">
         <v>10</v>
@@ -2535,7 +2550,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:10">
       <c r="A13" s="44"/>
       <c r="B13" s="14">
         <v>45007</v>
@@ -2630,7 +2645,7 @@
       <c r="I18" s="45"/>
       <c r="J18" s="47"/>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:10">
       <c r="A19" s="5"/>
       <c r="B19" s="6">
         <v>45007</v>
@@ -2645,7 +2660,7 @@
       <c r="F19" s="7"/>
       <c r="G19" s="9"/>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:10">
       <c r="A20" s="5"/>
       <c r="B20" s="6">
         <v>44995</v>
@@ -2660,7 +2675,7 @@
       <c r="F20" s="7"/>
       <c r="G20" s="9"/>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:10">
       <c r="A21" s="5"/>
       <c r="B21" s="6">
         <v>44995</v>
@@ -2675,7 +2690,7 @@
       <c r="F21" s="7"/>
       <c r="G21" s="9"/>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:10">
       <c r="A22" s="20"/>
       <c r="B22" s="29"/>
       <c r="C22" s="20"/>
@@ -2686,7 +2701,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:10">
       <c r="A23" s="43"/>
       <c r="B23" s="42">
         <v>45037</v>
@@ -2701,7 +2716,7 @@
       <c r="F23" s="15"/>
       <c r="G23" s="9"/>
     </row>
-    <row r="24" spans="1:7">
+    <row r="24" spans="1:10">
       <c r="A24" s="5"/>
       <c r="B24" s="6">
         <v>44988</v>
@@ -2716,7 +2731,7 @@
       <c r="F24" s="7"/>
       <c r="G24" s="9"/>
     </row>
-    <row r="25" spans="1:7">
+    <row r="25" spans="1:10">
       <c r="A25" s="5"/>
       <c r="B25" s="6">
         <v>44988</v>
@@ -2731,7 +2746,7 @@
       <c r="F25" s="7"/>
       <c r="G25" s="9"/>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:10">
       <c r="A26" s="30"/>
       <c r="B26" s="30" t="s">
         <v>10</v>
@@ -2746,7 +2761,7 @@
       <c r="F26" s="31"/>
       <c r="G26" s="9"/>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:10">
       <c r="A27" s="5"/>
       <c r="B27" s="6">
         <v>45012</v>
@@ -2761,7 +2776,7 @@
       <c r="F27" s="7"/>
       <c r="G27" s="9"/>
     </row>
-    <row r="28" spans="1:7">
+    <row r="28" spans="1:10">
       <c r="A28" s="11"/>
       <c r="B28" s="14">
         <v>45027</v>
@@ -2778,7 +2793,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="29" spans="1:7">
+    <row r="29" spans="1:10">
       <c r="A29" s="20"/>
       <c r="B29" s="29"/>
       <c r="C29" s="20"/>
@@ -2789,7 +2804,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="30" spans="1:7">
+    <row r="30" spans="1:10">
       <c r="A30" s="20"/>
       <c r="B30" s="34"/>
       <c r="C30" s="20"/>
@@ -2801,7 +2816,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G30">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:G30" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2814,9 +2829,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="15.7272727272727" customWidth="1"/>
+    <col min="1" max="1" width="15.7256637168142" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
@@ -2835,7 +2850,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="8.72566371681416" defaultRowHeight="13.5"/>
   <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -2846,7 +2861,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="8.72566371681416" defaultRowHeight="13.5"/>
   <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -2857,7 +2872,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="8.72566371681416" defaultRowHeight="13.5"/>
   <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -2868,14 +2883,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:H35"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="7"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="29.1090909090909" customWidth="1"/>
+    <col min="1" max="1" width="29.1061946902655" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="4" width="27.1090909090909" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="27.1090909090909" customWidth="1"/>
-    <col min="6" max="7" width="10.1090909090909" style="1" customWidth="1"/>
-    <col min="8" max="8" width="16.1090909090909" customWidth="1"/>
+    <col min="3" max="4" width="27.1061946902655" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="27.1061946902655" customWidth="1"/>
+    <col min="6" max="7" width="10.1061946902655" style="1" customWidth="1"/>
+    <col min="8" max="8" width="16.1061946902655" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -3438,7 +3453,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:8">
       <c r="A34" s="35"/>
       <c r="B34" s="36"/>
       <c r="C34" s="36"/>
@@ -3448,7 +3463,7 @@
       </c>
       <c r="F34" s="37"/>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:8">
       <c r="A35" s="38"/>
       <c r="B35" s="36"/>
       <c r="C35" s="36"/>
@@ -3459,7 +3474,7 @@
       <c r="F35" s="37"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H35">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H35" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>